<commit_message>
Begin loop over works
</commit_message>
<xml_diff>
--- a/Lingvistik_proj/lingvistik.xlsx
+++ b/Lingvistik_proj/lingvistik.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2285,6 +2285,1834 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This friend, and Sir Walter, did not marry, whatever might have been
+anticipated on that head by their acquaintance.  </t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As the head of the house, he felt that
+he ought to have been consulted, especially after taking the young man
+so publicly by the hand; "For they must have been seen together,"
+he observed, "once at Tattersall's, and twice in the lobby of
+the House of Commons."  </t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>We must be serious and decided; for after all, the person who
+has contracted debts must pay them; and though a great deal is due to
+the feelings of the gentleman, and the head of a house, like your father,
+there is still more due to the character of an honest man.</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">He was not only to quit his home,
+but to see it in the hands of others; a trial of fortitude,
+which stronger heads than Sir Walter's have found too much.
+</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>heads</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">It is a pity they are not knocked
+on the head at once, before they reach Admiral Baldwin's age."
+"Nay, Sir Walter," cried Mrs Clay, "this is being severe indeed.
+</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>She was quite easy on that head, and consequently
+full of strength and courage, till for a moment electrified by
+Mrs Croft's suddenly saying,--
+"It was you, and not your sister, I find, that my brother had
+the pleasure of being acquainted with, when he was in this country.</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">When the Crofts called this morning,
+(they called here afterwards, did not they?), they happened to say,
+that her brother, Captain Wentworth, is just returned to England,
+or paid off, or something, and is coming to see them almost directly;
+and most unluckily it came into mamma's head, when they were gone,
+that Wentworth, or something very like it, was the name of
+poor Richard's captain at one time; I do not know when or where,
+but a great while before he died, poor fellow!  </t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">And upon looking over
+his letters and things, she found it was so, and is perfectly sure
+that this must be the very man, and her head is quite full of it,
+and of poor Richard!  </t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">And in short,
+he had looked and said everything with such exquisite grace,
+that they could assure them all, their heads were both turned by him;
+and off they ran, quite as full of glee as of love, and apparently
+more full of Captain Wentworth than of little Charles.
+</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>heads</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">He was rich, and being turned on shore,
+fully intended to settle as soon as he could be properly tempted;
+actually looking round, ready to fall in love with all the speed
+which a clear head and a quick taste could allow.  </t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"
+"Charles may say what he pleases," cried Mary to Anne, as soon as
+he was out of the room, "but it would be shocking to have Henrietta
+marry Charles Hayter; a very bad thing for her, and still worse
+for me; and therefore it is very much to be wished that Captain Wentworth
+may soon put him quite out of her head, and I have very little doubt
+that he has.  </t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">She hoped, on turning her head,
+to see the master of the house; but it proved to be one
+much less calculated for making matters easy--Charles Hayter,
+probably not at all better pleased by the sight of Captain Wentworth
+than Captain Wentworth had been by the sight of Anne.
+</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In another moment, however, she found herself in the state of
+being released from him; some one was taking him from her,
+though he had bent down her head so much, that his little sturdy hands
+were unfastened from around her neck, and he was resolutely borne away,
+before she knew that Captain Wentworth had done it.
+</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mary had shewn herself disobliging to him,
+and was now to reap the consequence, which consequence was
+his dropping her arm almost every moment to cut off the heads
+of some nettles in the hedge with his switch; and when Mary began
+to complain of it, and lament her being ill-used, according to custom,
+in being on the hedge side, while Anne was never incommoded on the other,
+he dropped the arms of both to hunt after a weasel which he had
+a momentary glance of, and they could hardly get him along at all.
+</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>heads</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">They went back to dress and dine; and so well had the scheme
+answered already, that nothing was found amiss; though its being
+"so entirely out of season," and the "no thoroughfare of Lyme,"
+and the "no expectation of company," had brought many apologies
+from the heads of the inn.
+</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>heads</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Captain Benwick listened attentively, and seemed grateful for
+the interest implied; and though with a shake of the head,
+and sighs which declared his little faith in the efficacy of any books
+on grief like his, noted down the names of those she recommended,
+and promised to procure and read them.
+</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The head had received a severe contusion, but he had seen greater injuries
+recovered from:  he was by no means hopeless; he spoke cheerfully.
+</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">There was no injury but to the head.
+</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A new sort of way this,
+for a young fellow to be making love, by breaking his mistress's head,
+is not it, Miss Elliot?  </t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is breaking a head and giving a plaster,
+truly!"
+Admiral Croft's manners were not quite of the tone to suit Lady Russell,
+but they delighted Anne.  </t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">They had left Louisa beginning to sit up;
+but her head, though clear, was exceedingly weak, and her nerves
+susceptible to the highest extreme of tenderness; and though
+she might be pronounced to be altogether doing very well,
+it was still impossible to say when she might be able to bear
+the removal home; and her father and mother, who must return
+in time to receive their younger children for the Christmas holidays,
+had hardly a hope of being allowed to bring her with them.
+</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>His head is full of some books that he is reading upon your recommendation,
+and he wants to talk to you about them; he has found out something or other
+in one of them which he thinks--oh!</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>His declining to be on cordial terms with the head of his family,
+has left a very strong impression in his disfavour with me.</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">He had not seen Louisa;
+and was so extremely fearful of any ill consequence to her
+from an interview, that he did not press for it at all; and,
+on the contrary, seemed to have a plan of going away for a week
+or ten days, till her head was stronger.  </t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In Lady Russell's view, it was perfectly natural that Mr Elliot,
+at a mature time of life, should feel it a most desirable object,
+and what would very generally recommend him among all sensible people,
+to be on good terms with the head of his family; the simplest process
+in the world of time upon a head naturally clear, and only erring
+in the heyday of youth.  </t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In Lady Russell's view, it was perfectly natural that Mr Elliot,
+at a mature time of life, should feel it a most desirable object,
+and what would very generally recommend him among all sensible people,
+to be on good terms with the head of his family; the simplest process
+in the world of time upon a head naturally clear, and only erring
+in the heyday of youth.  </t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The neglect
+had been visited on the head of the sinner; for when poor Lady Elliot
+died herself, no letter of condolence was received at Kellynch,
+and, consequently, there was but too much reason to apprehend
+that the Dalrymples considered the relationship as closed.
+</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">My cousin Anne shakes her head.
+</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anne heard her,
+and made no violent exclamations; she only smiled, blushed,
+and gently shook her head.
+</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How Charles could take such a thing into his head was always
+incomprehensible to me.  </t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">At last, Lady Russell drew back her head.  </t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I should like to know why you imagine I am?"
+Mrs Smith looked at her again, looked earnestly, smiled,
+shook her head, and exclaimed--
+"Now, how I do wish I understood you!  </t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>"Do tell me how it first came into your head.</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"
+"It first came into my head," replied Mrs Smith, "upon finding how much
+you were together, and feeling it to be the most probable thing
+in the world to be wished for by everybody belonging to either of you;
+and you may depend upon it that all your acquaintance have disposed of you
+in the same way.  </t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>He was full of `to-morrow,' and it is very evident that I have been
+full of it too, ever since I entered the house, and learnt the extension
+of your plan and all that had happened, or my seeing him could never have
+gone so entirely out of my head.</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Her faith was plighted,
+and Mr Elliot's character, like the Sultaness Scheherazade's head,
+must live another day.
+</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">She felt its application
+to herself, felt it in a nervous thrill all over her; and at the same
+moment that her eyes instinctively glanced towards the distant table,
+Captain Wentworth's pen ceased to move, his head was raised, pausing,
+listening, and he turned round the next instant to give a look,
+one quick, conscious look at her.
+</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">He looked at her
+with a smile, and a little motion of the head, which expressed,
+"Come to me, I have something to say;" and the unaffected,
+easy kindness of manner which denoted the feelings of an older acquaintance
+than he really was, strongly enforced the invitation.  </t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The chair was earnestly protested against,
+and Mrs Musgrove, who thought only of one sort of illness,
+having assured herself with some anxiety, that there had been no fall
+in the case; that Anne had not at any time lately slipped down,
+and got a blow on her head; that she was perfectly convinced of having
+had no fall; could part with her cheerfully, and depend on
+finding her better at night.
+</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">When any two young people
+take it into their heads to marry, they are pretty sure by perseverance
+to carry their point, be they ever so poor, or ever so imprudent,
+or ever so little likely to be necessary to each other's ultimate comfort.
+</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>heads</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>gutenberg</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>austen-persuasion.txt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
First handling of works in NLTK and added form gutenberg nlkt path working
</commit_message>
<xml_diff>
--- a/Lingvistik_proj/lingvistik.xlsx
+++ b/Lingvistik_proj/lingvistik.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,10 +473,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">"That is what you have in your head,
-I know--and what you would certainly say if my father were not by."
-"I believe it is very true, my dear, indeed," said Mr. Woodhouse,
-with a sigh.  </t>
+          <t>Mrs. Norris was often observing to the others that she could not get her poor sister and her family out of her head, and that, much as they had all done for her, she seemed to be wanting to do more; and at length she could not but own it to be her wish that poor Mrs. Price should be relieved from the charge and expense of one child entirely out of her great number.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -506,22 +503,19 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">"But, Mr. Knightley, she is really very sorry to lose poor Miss Taylor,
-and I am sure she _will_ miss her more than she thinks for."
-Emma turned away her head, divided between tears and smiles.
-</t>
+          <t>She hung her head and answered hesitatingly, âshe did not know; she had not any paper.â  âIf that be all your difficulty, I will furnish you with paper and every other material, and you may write your letter whenever you choose.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -551,20 +545,19 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"
-Mr. Knightley shook his head at her.  </t>
+          <t>He had been visiting a friend in the neighbouring county, and that friend having recently had his grounds laid out by an improver, Mr. Rushworth was returned with his head full of the subject, and very eager to be improving his own place in the same way; and though not saying much to the purpose, could talk of nothing else.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -594,20 +587,19 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mr. Elton was the very person fixed on by Emma for driving
-the young farmer out of Harriet's head.  </t>
+          <t xml:space="preserve">No wonder her head aches.â  Mrs. Norris was talking to Julia, and did not hear.  </t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -637,20 +629,19 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">There is health, not merely in her bloom, but in her air, her head,
-her glance.  </t>
+          <t xml:space="preserve">As she leant on the sofa, to which she had retreated that she might not be seen, the pain of her mind had been much beyond that in her head; and the sudden change which Edmundâs kindness had then occasioned, made her hardly know how to support herself.     </t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -680,19 +671,19 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">He had nestled down his head most conveniently.  </t>
+          <t>The situation of the house excluded the possibility of much prospect from any of the rooms; and while Fanny and some of the others were attending Mrs. Rushworth, Henry Crawford was looking grave and shaking his head at the windows.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -722,25 +713,24 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vanity working on a weak head,
-produces every sort of mischief.  </t>
+          <t>âIt must do the heads of the family a great deal of good to force all the poor housemaids and footmen to leave business and pleasure, and say their prayers here twice a day, while they are inventing excuses themselves for staying away.â  â_That_ is hardly Fannyâs idea of a family assembling,â said Edmund.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>heads</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -765,27 +755,24 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Miss Nash, head-teacher at Mrs. Goddard's,
-had written out at least three hundred; and Harriet, who had taken
-the first hint of it from her, hoped, with Miss Woodhouse's help,
-to get a great many more.  </t>
+          <t>The young Mrs. Eleanors and Mrs. Bridgetsâstarched up into seeming piety, but with heads full of something very differentâespecially if the poor chaplain were not worth looking atâand, in those days, I fancy parsons were very inferior even to what they are now.â  For a few moments she was unanswered.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>heads</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -810,22 +797,19 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">They had not been long seated and composed when Mr. Woodhouse,
-with a melancholy shake of the head and a sigh, called his daughter's
-attention to the sad change at Hartfield since she had been there last.
-</t>
+          <t>âFor if,â said he, with the sort of self-evident proposition which many a clearer head does not always avoid, âwe are _too_</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -855,25 +839,19 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">"
-"I am sorry to hear you say so, sir; but I assure you, excepting those
-little nervous head-aches and palpitations which I am never entirely
-free from anywhere, I am quite well myself; and if the children were
-rather pale before they went to bed, it was only because they were
-a little more tired than usual, from their journey and the happiness
-of coming.  </t>
+          <t>He must not head mobs, or set the ton in dress.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -903,22 +881,19 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Ah!" said Mr. Woodhouse, shaking his head and fixing his eyes on
-her with tender concern.--The ejaculation in Emma's ear expressed,
-"Ah! there is no end of the sad consequences of your going to
-South End.  </t>
+          <t xml:space="preserve">But when my aunt has got a fancy in her head, nothing can stop her.â     CHAPTER XIII   </t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -948,25 +923,19 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">How they were all to be conveyed, he would have made a difficulty
-if he could, but as his son and daughter's carriage and horses
-were actually at Hartfield, he was not able to make more than
-a simple question on that head; it hardly amounted to a doubt;
-nor did it occupy Emma long to convince him that they might in one
-of the carriages find room for Harriet also.
-</t>
+          <t>He came on the wings of disappointment, and with his head full of acting, for it had been a theatrical party; and the play in which he had borne a part was within two days of representation, when the sudden death of one of the nearest connexions of the family had destroyed the scheme and dispersed the performers.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -996,26 +965,19 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">But he had fancied her in love with him; that evidently must
-have been his dependence; and after raving a little about the
-seeming incongruity of gentle manners and a conceited head,
-Emma was obliged in common honesty to stop and admit that her own
-behaviour to him had been so complaisant and obliging, so full of
-courtesy and attention, as (supposing her real motive unperceived)
-might warrant a man of ordinary observation and delicacy,
-like Mr. Elton, in fancying himself a very decided favourite.  </t>
+          <t xml:space="preserve">Edmund smiled and shook his head.  </t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1045,27 +1007,19 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Harriet said, "very true," and she "would not think about it;"
-but still she talked of it--still she could talk of nothing else;
-and Emma, at last, in order to put the Martins out of her head,
-was obliged to hurry on the news, which she had meant to give
-with so much tender caution; hardly knowing herself whether
-to rejoice or be angry, ashamed or only amused, at such a state
-of mind in poor Harriet--such a conclusion of Mr. Elton's importance
-with her!
-</t>
+          <t>There_ would be the greatest indecorum, I think.â  âDo you imagine that I could have such an idea in my head?</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1095,22 +1049,19 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">"
-He shook his head and laughed.--"I cannot separate Miss Fairfax
-and her complexion."
-</t>
+          <t>There should always be one steady head to superintend so many young ones.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1140,29 +1091,24 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Yes, and what you told me on that head, confirmed an idea which I
-had entertained before.--I do not mean to reflect upon the good
-intentions of either Mr. Dixon or Miss Fairfax, but I cannot help
-suspecting either that, after making his proposals to her friend,
-he had the misfortune to fall in love with _her_, or that he became
-conscious of a little attachment on her side.  </t>
+          <t>I knew what all this meant, for the servantsâ dinner-bell was ringing at the very moment over our heads; and as I hate such encroaching people (the Jacksons are very encroaching, I have always said so: just the sort of people to get all they can), I said to the boy directly (a great lubberly fellow of ten years old, you know, who ought to be ashamed of himself), â_Iâll_ take the boards to your father, Dick, so get you home again as fast as you can.â The boy looked very silly, and turned away without offering a word, for I believe I might speak pretty sharp; and I dare say it will cure him of coming marauding about the house for one while.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>heads</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1187,22 +1133,19 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Well," said Mrs. Weston, smiling, "you give him credit for
-more simple, disinterested benevolence in this instance than I do;
-for while Miss Bates was speaking, a suspicion darted into my head,
-and I have never been able to get it out again.  </t>
+          <t xml:space="preserve">Mr. Yates, who was trying to make himself agreeable to Julia, found her gloom less impenetrable on any topic than that of his regret at her secession from their company; and Mr. Rushworth, having only his own part and his own dress in his head, had soon talked away all that could be said of either.  </t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1232,19 +1175,19 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do not put it into his head.  </t>
+          <t>Sleeping or waking, my head has been full of this matter all night.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1274,21 +1217,19 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">"
-He shook his head with a smile, and looked as if he had very little
-doubt and very little mercy.  </t>
+          <t>I admire your little establishment exceedingly; and as soon as I am gone, you will empty your head of all this nonsense of acting, and sit comfortably down to your table.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1318,21 +1259,19 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">But Emma
-still shook her head in steady scepticism.
-</t>
+          <t>He has a fine dignified manner, which suits the head of such a house, and keeps everybody in their place.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1362,22 +1301,19 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">When his letter to Mrs. Weston arrived, Emma had the perusal of it;
-and she read it with a degree of pleasure and admiration which made
-her at first shake her head over her own sensations, and think she
-had undervalued their strength.  </t>
+          <t>I will ask Sir Thomas, as soon as he comes in, whether I can do without her.â  âAs you please, maâam, on that head; but I meant my fatherâs opinion as to the _propriety_ of the invitationâs being accepted or not; and I think he will consider it a right thing by Mrs. Grant, as well as by Fanny, that being the _first_ invitation it should be accepted.â  âI do not know.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1407,21 +1343,19 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warmth and tenderness of heart, with an affectionate, open manner,
-will beat all the clearness of head in the world, for attraction,
-I am sure it will.  </t>
+          <t xml:space="preserve">Mrs. Grant thinks it a civility due to _us_ to take a little notice of you, or else it would never have come into her head, and you may be very certain that, if your cousin Julia had been at home, you would not have been asked at all.â  Mrs. Norris had now so ingeniously done away all Mrs. Grantâs part of the favour, that Fanny, who found herself expected to speak, could only say that she was very much obliged to her aunt Bertram for sparing her, and that she was endeavouring to put her auntâs evening work in such a state as to prevent her being missed.  </t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1451,25 +1385,24 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dear Harriet!--I would not change you for the clearest-headed,
-longest-sighted, best-judging female breathing.  </t>
+          <t xml:space="preserve">He honoured the warm-hearted, blunt fondness of the young sailor, which led him to say, with his hands stretched towards Fannyâs head, âDo you know, I begin to like that queer fashion already, though when I first heard of such things being done in England, I could not believe it; and when Mrs. Brown, and the other women at the Commissionerâs at Gibraltar, appeared in the same trim, I thought they were mad; but Fanny can reconcile me to anythingâ; and saw, with lively admiration, the glow of Fannyâs cheek, the brightness of her eye, the deep interest, the absorbed attention, while her brother was describing any of the imminent hazards, or terrific scenes, which such a period at sea must supply.  </t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>headed</t>
+          <t>head</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1494,20 +1427,19 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">"
-"No, indeed, I have no doubts at all on that head.  </t>
+          <t>With something of consciousness he shook his head at his sister, and laughingly replied, âI cannot say there was much done at Sotherton; but it was a hot day, and we were all walking after each other, and bewildered.â As soon as a general buzz gave him shelter, he added, in a low voice, directed solely at Fanny, âI should be sorry to have my powers of _planning_ judged of by the day at Sotherton.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1537,30 +1469,29 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">No--till Cole alluded to my supposed attachment,
-it had never entered my head.  </t>
+          <t xml:space="preserve">I do not exactly know the distance, but when you get back to Portsmouth, if it is not very far off, you ought to go over and pay your respects to them; and I could send a little parcel by you that I want to get conveyed to your cousins.â  âI should be very happy, aunt; but Brighton is almost by Beachey Head; and if I could get so far, I could not expect to be welcome in such a smart place as thatâpoor scrubby midshipman as I am.â  Mrs. Norris was beginning an eager assurance of the affability he might depend on, when she was stopped by Sir Thomasâs saying with authority, âI do not advise your going to Brighton, William, as I trust you may soon have more convenient opportunities of meeting; but my daughters would be happy to see their cousins anywhere; and you will find Mr. Rushworth most sincerely disposed to regard all the connexions of our family as his own.â  âI would rather find him private secretary to the First Lord than anything else,â was Williamâs only answer, in an undervoice, not meant to reach far, and the subject dropped.  </t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>Head</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>Head</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1580,22 +1511,19 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">"
-"I not aware!" said Jane, shaking her head; "dear Mrs. Elton,
-who can have thought of it as I have done?"
-</t>
+          <t>Invitations were sent with despatch, and many a young lady went to bed that night with her head full of happy cares as well as Fanny.</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1625,25 +1553,24 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">"She has taken it into her head that Enscombe is too
-cold for her.  </t>
+          <t>But Miss Crawford persevered, and argued the case with so much affectionate earnestness through all the heads of William and the cross, and the ball, and herself, as to be finally successful.</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>heads</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1668,21 +1595,19 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">She was not yet dancing; she was working her way
-up from the bottom, and had therefore leisure to look around,
-and by only turning her head a little she saw it all.  </t>
+          <t>Starting and looking up, she saw, across the lobby she had just reached, Edmund himself, standing at the head of a different staircase.</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1712,21 +1637,19 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">He shook his head; but there was a smile of indulgence with it,
-and he only said,
-"I shall not scold you.  </t>
+          <t xml:space="preserve">but that she was really pleased to have Fanny admired; but she was so much more struck with her own kindness in sending Chapman to her, that she could not get it out of her head.  </t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1756,35 +1679,24 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">How the trampers might have behaved, had the young ladies been
-more courageous, must be doubtful; but such an invitation for attack
-could not be resisted; and Harriet was soon assailed by half a
-dozen children, headed by a stout woman and a great boy, all clamorous,
-and impertinent in look, though not absolutely in word.--More and
-more frightened, she immediately promised them money, and taking out
-her purse, gave them a shilling, and begged them not to want more,
-or to use her ill.--She was then able to walk, though but slowly,
-and was moving away--but her terror and her purse were too tempting,
-and she was followed, or rather surrounded, by the whole gang,
-demanding more.
-</t>
+          <t>You will both find your good in it.â  âIt was bad, very bad in me against such a creature; but I did not know her then; and she shall have no reason to lament the hour that first put it into my head.</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>headed</t>
+          <t>head</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1809,19 +1721,19 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>And how could it possibly come into your head?</t>
+          <t>She would not stir farther from the East room than the head of the great staircase, till she had satisfied herself of Mr. Crawfordâs having left the house; but when convinced of his being gone, she was eager to go down and be with her uncle, and have all the happiness of his joy as well as her own, and all the benefit of his information or his conjectures as to what would now be Williamâs destination.</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1851,26 +1763,19 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">And poor John's son came to talk to Mr. Elton
-about relief from the parish; he is very well to do himself,
-you know, being head man at the Crown, ostler, and every thing
-of that sort, but still he cannot keep his father without some help;
-and so, when Mr. Elton came back, he told us what John ostler
-had been telling him, and then it came out about the chaise having
-been sent to Randalls to take Mr. Frank Churchill to Richmond.
-</t>
+          <t>You must have observed his attentions; and though you always received them very properly (I have no accusation to make on that head), I never perceived them to be unpleasant to you.</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1900,24 +1805,19 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emma's colour was heightened by this unjust praise; and with a smile,
-and shake of the head, which spoke much, she looked at Mr. Knightley.--
-It seemed as if there were an instantaneous impression in her favour,
-as if his eyes received the truth from her's, and all that had
-passed of good in her feelings were at once caught and honoured.--
-He looked at her with a glow of regard.  </t>
+          <t xml:space="preserve">And I do not know that I should be fond of preaching often; now and then, perhaps once or twice in the spring, after being anxiously expected for half a dozen Sundays together; but not for a constancy; it would not do for a constancy.â  Here Fanny, who could not but listen, involuntarily shook her head, and Crawford was instantly by her side again, entreating to know her meaning; and as Edmund perceived, by his drawing in a chair, and sitting down close by her, that it was to be a very thorough attack, that looks and undertones were to be well tried, he sank as quietly as possible into a corner, turned his back, and took up a newspaper, very sincerely wishing that dear little Fanny might be persuaded into explaining away that shake of the head to the satisfaction of her ardent lover; and as earnestly trying to bury every sound of the business from himself in murmurs of his own, over the various advertisements of âA most desirable Estate in South Walesâ; âTo Parents and Guardiansâ; and a âCapital seasonâd Hunter.â  Fanny, meanwhile, vexed with herself for not having been as motionless as she was speechless, and grieved to the heart to see Edmundâs arrangements, was trying by everything in the power of her modest, gentle nature, to repulse Mr. Crawford, and avoid both his looks and inquiries; and he, unrepulsable, was persisting in both.  </t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1947,23 +1847,19 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Even Mr. Weston shook his head, and looked solemn, and said,
-"Ah! poor woman, who would have thought it!" and resolved, that his
-mourning should be as handsome as possible; and his wife sat sighing
-and moralising over her broad hems with a commiseration and good sense,
-true and steady.  </t>
+          <t xml:space="preserve">And I do not know that I should be fond of preaching often; now and then, perhaps once or twice in the spring, after being anxiously expected for half a dozen Sundays together; but not for a constancy; it would not do for a constancy.â  Here Fanny, who could not but listen, involuntarily shook her head, and Crawford was instantly by her side again, entreating to know her meaning; and as Edmund perceived, by his drawing in a chair, and sitting down close by her, that it was to be a very thorough attack, that looks and undertones were to be well tried, he sank as quietly as possible into a corner, turned his back, and took up a newspaper, very sincerely wishing that dear little Fanny might be persuaded into explaining away that shake of the head to the satisfaction of her ardent lover; and as earnestly trying to bury every sound of the business from himself in murmurs of his own, over the various advertisements of âA most desirable Estate in South Walesâ; âTo Parents and Guardiansâ; and a âCapital seasonâd Hunter.â  Fanny, meanwhile, vexed with herself for not having been as motionless as she was speechless, and grieved to the heart to see Edmundâs arrangements, was trying by everything in the power of her modest, gentle nature, to repulse Mr. Crawford, and avoid both his looks and inquiries; and he, unrepulsable, was persisting in both.  </t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1993,29 +1889,19 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">What has it been
-but a system of hypocrisy and deceit,--espionage, and treachery?--
-To come among us with professions of openness and simplicity;
-and such a league in secret to judge us all!--Here have we been,
-the whole winter and spring, completely duped, fancying ourselves
-all on an equal footing of truth and honour, with two people in the
-midst of us who may have been carrying round, comparing and sitting
-in judgment on sentiments and words that were never meant for both
-to hear.--They must take the consequence, if they have heard each
-other spoken of in a way not perfectly agreeable!"
-"I am quite easy on that head," replied Mrs. Weston.  </t>
+          <t>âWhat did that shake of the head mean?â said he.</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2045,27 +1931,19 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">How to understand the deceptions she had been thus practising
-on herself, and living under!--The blunders, the blindness of her
-own head and heart!--she sat still, she walked about, she tried her
-own room, she tried the shrubbery--in every place, every posture,
-she perceived that she had acted most weakly; that she had been imposed
-on by others in a most mortifying degree; that she had been imposing
-on herself in a degree yet more mortifying; that she was wretched,
-and should probably find this day but the beginning of wretchedness.
-</t>
+          <t xml:space="preserve">What did that shake of the head mean?â  </t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2095,26 +1973,19 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">"
-When he came to Miss Woodhouse, he was obliged to read the whole
-of it aloud--all that related to her, with a smile; a look;
-a shake of the head; a word or two of assent, or disapprobation;
-or merely of love, as the subject required; concluding, however,
-seriously, and, after steady reflection, thus--
-"Very bad--though it might have been worse.--Playing a most
-dangerous game.  </t>
+          <t>âYou shook your head at my acknowledging that I should not like to engage in the duties of a clergyman always for a constancy.</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2144,27 +2015,24 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>"
-And again, on Emma's merely turning her head to look
-at Mrs. Bates's knitting, she added, in a half whisper,
-"I mentioned no _names_, you will observe.--Oh!</t>
+          <t>The solemn procession, headed by Baddeley, of tea-board, urn, and cake-bearers, made its appearance, and delivered her from a grievous imprisonment of body and mind.</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>headed</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2189,21 +2057,19 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Observe her eyes, as she is looking up at my father.--
-You will be glad to hear (inclining his head, and whispering seriously)
-that my uncle means to give her all my aunt's jewels.  </t>
+          <t>She immediately shook her head at Fanny with arch, yet affectionate reproach, and taking her hand, seemed hardly able to help beginning directly.</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2233,20 +2099,19 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">I am resolved to have some in an ornament for the head.
-</t>
+          <t>He is just what the head of such a family should be.</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2276,20 +2141,19 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">This friend, and Sir Walter, did not marry, whatever might have been
-anticipated on that head by their acquaintance.  </t>
+          <t>I am ashamed to say that it had never entered my head, but I was delighted to act on his proposal for both your sakes.â  âI will not say,â replied Fanny, âthat I was not half afraid at the time of its being so, for there was something in your look that frightened me, but not at first; I was as unsuspicious of it at firstâindeed, indeed I was.</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2319,23 +2183,19 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">As the head of the house, he felt that
-he ought to have been consulted, especially after taking the young man
-so publicly by the hand; "For they must have been seen together,"
-he observed, "once at Tattersall's, and twice in the lobby of
-the House of Commons."  </t>
+          <t>I am sure it is not in womanâs nature to refuse such a triumph.â  Fanny shook her head.</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2365,22 +2225,19 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>We must be serious and decided; for after all, the person who
-has contracted debts must pay them; and though a great deal is due to
-the feelings of the gentleman, and the head of a house, like your father,
-there is still more due to the character of an honest man.</t>
+          <t xml:space="preserve">She must say that she had more than half a mind to go with the young people; it would be such an indulgence to her; she had not seen her poor dear sister Price for more than twenty years; and it would be a help to the young people in their journey to have her older head to manage for them; and she could not help thinking her poor dear sister Price would feel it very unkind of her not to come by such an opportunity.  </t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2410,27 +2267,24 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">He was not only to quit his home,
-but to see it in the hands of others; a trial of fortitude,
-which stronger heads than Sir Walter's have found too much.
-</t>
+          <t xml:space="preserve">The solitary candle was held between himself and the paper, without any reference to her possible convenience; but she had nothing to do, and was glad to have the light screened from her aching head, as she sat in bewildered, broken, sorrowful contemplation.  </t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>heads</t>
+          <t>head</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2455,22 +2309,19 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">It is a pity they are not knocked
-on the head at once, before they reach Admiral Baldwin's age."
-"Nay, Sir Walter," cried Mrs Clay, "this is being severe indeed.
-</t>
+          <t>Fannyâs spirit was as much refreshed as her body; her head and heart were soon the better for such well-timed kindness.</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2500,23 +2351,19 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>She was quite easy on that head, and consequently
-full of strength and courage, till for a moment electrified by
-Mrs Croft's suddenly saying,--
-"It was you, and not your sister, I find, that my brother had
-the pleasure of being acquainted with, when he was in this country.</t>
+          <t>Such was the home which was to put Mansfield out of her head, and teach her to think of her cousin Edmund with moderated feelings.</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2546,26 +2393,19 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">When the Crofts called this morning,
-(they called here afterwards, did not they?), they happened to say,
-that her brother, Captain Wentworth, is just returned to England,
-or paid off, or something, and is coming to see them almost directly;
-and most unluckily it came into mamma's head, when they were gone,
-that Wentworth, or something very like it, was the name of
-poor Richard's captain at one time; I do not know when or where,
-but a great while before he died, poor fellow!  </t>
+          <t>The promised notification was hanging over her head.</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2595,22 +2435,19 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">And upon looking over
-his letters and things, she found it was so, and is perfectly sure
-that this must be the very man, and her head is quite full of it,
-and of poor Richard!  </t>
+          <t>Luckily there is no distinction of dress nowadays to tell tales, butâbutâbut Yours affectionately.â  âI had almost forgot (it was Edmundâs fault: he gets into my head more than does me good)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2640,29 +2477,24 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">And in short,
-he had looked and said everything with such exquisite grace,
-that they could assure them all, their heads were both turned by him;
-and off they ran, quite as full of glee as of love, and apparently
-more full of Captain Wentworth than of little Charles.
-</t>
+          <t>To all she must have saved some trouble of head or hand; and were it only in supporting the spirits of her aunt Bertram, keeping her from the evil of solitude, or the still greater evil of a restless, officious companion, too apt to be heightening danger in order to enhance her own importance, her being there would have been a general good.</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>heads</t>
+          <t>head</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2687,22 +2519,19 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">He was rich, and being turned on shore,
-fully intended to settle as soon as he could be properly tempted;
-actually looking round, ready to fall in love with all the speed
-which a clear head and a quick taste could allow.  </t>
+          <t xml:space="preserve">She could still think of little else all the morning; but, when her father came back in the afternoon with the daily newspaper as usual, she was so far from expecting any elucidation through such a channel that the subject was for a moment out of her head.  </t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2732,25 +2561,19 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">"
-"Charles may say what he pleases," cried Mary to Anne, as soon as
-he was out of the room, "but it would be shocking to have Henrietta
-marry Charles Hayter; a very bad thing for her, and still worse
-for me; and therefore it is very much to be wished that Captain Wentworth
-may soon put him quite out of her head, and I have very little doubt
-that he has.  </t>
+          <t>She sat in a blaze of oppressive heat, in a cloud of moving dust, and her eyes could only wander from the walls, marked by her fatherâs head, to the table cut and notched by her brothers, where stood the tea-board never thoroughly cleaned, the cups and saucers wiped in streaks, the milk a mixture of motes floating in thin blue, and the bread and butter growing every minute more greasy than even Rebeccaâs hands had first produced it.</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2780,24 +2603,19 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">She hoped, on turning her head,
-to see the master of the house; but it proved to be one
-much less calculated for making matters easy--Charles Hayter,
-probably not at all better pleased by the sight of Captain Wentworth
-than Captain Wentworth had been by the sight of Anne.
-</t>
+          <t xml:space="preserve">They lived together; and when Dr. Grant had brought on apoplexy and death, by three great institutionary dinners in one week, they still lived together; for Mary, though perfectly resolved against ever attaching herself to a younger brother again, was long in finding among the dashing representatives, or idle heir-apparents, who were at the command of her beauty, and her Â£20,000, any one who could satisfy the better taste she had acquired at Mansfield, whose character and manners could authorise a hope of the domestic happiness she had there learned to estimate, or put Edmund Bertram sufficiently out of her head.  </t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2827,29 +2645,24 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Mansfield Park.txt</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">In another moment, however, she found herself in the state of
-being released from him; some one was taking him from her,
-though he had bent down her head so much, that his little sturdy hands
-were unfastened from around her neck, and he was resolutely borne away,
-before she knew that Captain Wentworth had done it.
-</t>
+          <t>A family of ten children will be always called a fine family, where there are heads and arms and legs enough for the number; but the Morlands had little other right to the word, for they were in general very plain, and Catherine, for many years of her life, as plain as any.</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>heads</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2874,32 +2687,24 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mary had shewn herself disobliging to him,
-and was now to reap the consequence, which consequence was
-his dropping her arm almost every moment to cut off the heads
-of some nettles in the hedge with his switch; and when Mary began
-to complain of it, and lament her being ill-used, according to custom,
-in being on the hedge side, while Anne was never incommoded on the other,
-he dropped the arms of both to hunt after a weasel which he had
-a momentary glance of, and they could hardly get him along at all.
-</t>
+          <t>how is my head, my dear?</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>heads</t>
+          <t>head</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2924,29 +2729,24 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">They went back to dress and dine; and so well had the scheme
-answered already, that nothing was found amiss; though its being
-"so entirely out of season," and the "no thoroughfare of Lyme,"
-and the "no expectation of company," had brought many apologies
-from the heads of the inn.
-</t>
+          <t xml:space="preserve">I must give one smirk, and then we may be rational again.â Catherine turned away her head, not knowing whether she might venture to laugh.  </t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>heads</t>
+          <t>head</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2971,24 +2771,19 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Captain Benwick listened attentively, and seemed grateful for
-the interest implied; and though with a shake of the head,
-and sighs which declared his little faith in the efficacy of any books
-on grief like his, noted down the names of those she recommended,
-and promised to procure and read them.
-</t>
+          <t>âWhat are you thinking of so earnestly?â said he, as they walked back to the ballroom; ânot of your partner, I hope, for, by that shake of the head, your meditations are not satisfactory.â  Catherine coloured, and said, âI was not thinking of anything.â  âThat is artful and deep, to be sure; but I had rather be told at once that you will not tell me.â  âWell then, I will not.â  âThank you; for now we shall soon be acquainted, as I am authorized to tease you on this subject whenever we meet, and nothing in the world advances intimacy so much.â  They danced again; and, when the assembly closed, parted, on the ladyâs side at least, with a strong inclination for continuing the acquaintance.</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3018,21 +2813,19 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">The head had received a severe contusion, but he had seen greater injuries
-recovered from:  he was by no means hopeless; he spoke cheerfully.
-</t>
+          <t xml:space="preserve">How proper Mr. Tilney might be as a dreamer or a lover had not yet perhaps entered Mr. Allenâs head, but that he was not objectionable as a common acquaintance for his young charge he was on inquiry satisfied; for he had early in the evening taken pains to know who her partner was, and had been assured of Mr. Tilneyâs being a clergyman, and of a very respectable family in Gloucestershire.   </t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3062,20 +2855,19 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">There was no injury but to the head.
-</t>
+          <t>But, my dearest Catherine, have you settled what to wear on your head to-night?</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3105,21 +2897,19 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">A new sort of way this,
-for a young fellow to be making love, by breaking his mistress's head,
-is not it, Miss Elliot?  </t>
+          <t>But guided only by what was simple and probable, it had never entered her head that Mr. Tilney could be married; he had not behaved, he had not talked, like the married men to whom she had been used; he had never mentioned a wife, and he had acknowledged a sister.</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3149,22 +2939,19 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">This is breaking a head and giving a plaster,
-truly!"
-Admiral Croft's manners were not quite of the tone to suit Lady Russell,
-but they delighted Anne.  </t>
+          <t>You know I never stand upon ceremony with such people.â  âLook at that young lady with the white beads round her head,â whispered Catherine, detaching her friend from James.</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3194,27 +2981,19 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">They had left Louisa beginning to sit up;
-but her head, though clear, was exceedingly weak, and her nerves
-susceptible to the highest extreme of tenderness; and though
-she might be pronounced to be altogether doing very well,
-it was still impossible to say when she might be able to bear
-the removal home; and her father and mother, who must return
-in time to receive their younger children for the Christmas holidays,
-had hardly a hope of being allowed to bring her with them.
-</t>
+          <t>What a head you have!</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3244,21 +3023,19 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>His head is full of some books that he is reading upon your recommendation,
-and he wants to talk to you about them; he has found out something or other
-in one of them which he thinks--oh!</t>
+          <t>Everything being then arranged, the servant who stood at the horseâs head was bid in an important voice âto let him go,â and off they went in the quietest manner imaginable, without a plunge or a caper, or anything like one.</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3288,20 +3065,19 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>His declining to be on cordial terms with the head of his family,
-has left a very strong impression in his disfavour with me.</t>
+          <t>Now, for instance, it was reckoned a remarkable thing, at the last party in my rooms, that upon an average we cleared about five pints a head.</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3331,23 +3107,19 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">He had not seen Louisa;
-and was so extremely fearful of any ill consequence to her
-from an interview, that he did not press for it at all; and,
-on the contrary, seemed to have a plan of going away for a week
-or ten days, till her head was stronger.  </t>
+          <t>What gown and what head-dress she should wear on the occasion became her chief concern.</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3377,24 +3149,19 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">In Lady Russell's view, it was perfectly natural that Mr Elliot,
-at a mature time of life, should feel it a most desirable object,
-and what would very generally recommend him among all sensible people,
-to be on good terms with the head of his family; the simplest process
-in the world of time upon a head naturally clear, and only erring
-in the heyday of youth.  </t>
+          <t>Confused by his notice, and blushing from the fear of its being excited by something wrong in her appearance, she turned away her head.</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3424,29 +3191,24 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">In Lady Russell's view, it was perfectly natural that Mr Elliot,
-at a mature time of life, should feel it a most desirable object,
-and what would very generally recommend him among all sensible people,
-to be on good terms with the head of his family; the simplest process
-in the world of time upon a head naturally clear, and only erring
-in the heyday of youth.  </t>
+          <t>You are to thank your brother and me for the scheme; it darted into our heads at breakfast-time, I verily believe at the same instant; and we should have been off two hours ago if it had not been for this detestable rain.</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>heads</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3471,24 +3233,19 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">The neglect
-had been visited on the head of the sinner; for when poor Lady Elliot
-died herself, no letter of condolence was received at Kellynch,
-and, consequently, there was but too much reason to apprehend
-that the Dalrymples considered the relationship as closed.
-</t>
+          <t>At the head of them she was met by Mr. Allen, who, on hearing the reason of their speedy return, said, âI am glad your brother had so much sense; I am glad you are come back.</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3518,20 +3275,19 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">My cousin Anne shakes her head.
-</t>
+          <t>I will prove myself a man, no less by the generosity of my soul than the clearness of my head.</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3561,22 +3317,19 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anne heard her,
-and made no violent exclamations; she only smiled, blushed,
-and gently shook her head.
-</t>
+          <t>You talked of expected horrors in Londonâand instead of instantly conceiving, as any rational creature would have done, that such words could relate only to a circulating library, she immediately pictured to herself a mob of three thousand men assembling in St. Georgeâs Fields, the Bank attacked, the Tower threatened, the streets of London flowing with blood, a detachment of the Twelfth Light Dragoons (the hopes of the nation) called up from Northampton to quell the insurgents, and the gallant Captain Frederick Tilney, in the moment of charging at the head of his troop, knocked off his horse by a brickbat from an upper window.</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3606,20 +3359,19 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">How Charles could take such a thing into his head was always
-incomprehensible to me.  </t>
+          <t>Let me only have the girl I like, say I, with a comfortable house over my head, and what care I for all the rest?</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3649,19 +3401,19 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">At last, Lady Russell drew back her head.  </t>
+          <t>after what you told him from me, how could he think of going to ask her?â  âI cannot take surprise to myself on that head.</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3691,22 +3443,19 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">I should like to know why you imagine I am?"
-Mrs Smith looked at her again, looked earnestly, smiled,
-shook her head, and exclaimed--
-"Now, how I do wish I understood you!  </t>
+          <t>My poor head, I had quite forgot it.</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3736,19 +3485,19 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>"Do tell me how it first came into your head.</t>
+          <t>You know he is over head and ears in love with you.â  âWith _me_, dear Isabella!â  âNay, my sweetest Catherine, this is being quite absurd!</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3778,24 +3527,19 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">"
-"It first came into my head," replied Mrs Smith, "upon finding how much
-you were together, and feeling it to be the most probable thing
-in the world to be wished for by everybody belonging to either of you;
-and you may depend upon it that all your acquaintance have disposed of you
-in the same way.  </t>
+          <t>âWhy do you put such things into my head?</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3825,22 +3569,19 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>He was full of `to-morrow,' and it is very evident that I have been
-full of it too, ever since I entered the house, and learnt the extension
-of your plan and all that had happened, or my seeing him could never have
-gone so entirely out of my head.</t>
+          <t>Catherine trembled from head to foot.</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3870,22 +3611,19 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Her faith was plighted,
-and Mr Elliot's character, like the Sultaness Scheherazade's head,
-must live another day.
-</t>
+          <t xml:space="preserve">In this there was surely something mysterious, and she indulged in the flattering suggestion for half a minute, till the possibility of the doorâs having been at first unlocked, and of being herself its fastener, darted into her head, and cost her another blush.  </t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3915,25 +3653,19 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">She felt its application
-to herself, felt it in a nervous thrill all over her; and at the same
-moment that her eyes instinctively glanced towards the distant table,
-Captain Wentworth's pen ceased to move, his head was raised, pausing,
-listening, and he turned round the next instant to give a look,
-one quick, conscious look at her.
-</t>
+          <t>At that instant a door underneath was hastily opened; someone seemed with swift steps to ascend the stairs, by the head of which she had yet to pass before she could gain the gallery.</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3963,23 +3695,19 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">He looked at her
-with a smile, and a little motion of the head, which expressed,
-"Come to me, I have something to say;" and the unaffected,
-easy kindness of manner which denoted the feelings of an older acquaintance
-than he really was, strongly enforced the invitation.  </t>
+          <t>He often expressed his uneasiness on this head, feared the sameness of every dayâs society and employments would disgust her with the place, wished the Lady Frasers had been in the country, talked every now and then of having a large party to dinner, and once or twice began even to calculate the number of young dancing people in the neighbourhood.</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4009,26 +3737,19 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">The chair was earnestly protested against,
-and Mrs Musgrove, who thought only of one sort of illness,
-having assured herself with some anxiety, that there had been no fall
-in the case; that Anne had not at any time lately slipped down,
-and got a blow on her head; that she was perfectly convinced of having
-had no fall; could part with her cheerfully, and depend on
-finding her better at night.
-</t>
+          <t>He has his vanities as well as Miss Thorpe, and the chief difference is, that, having a stronger head, they have not yet injured himself.</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4058,58 +3779,264 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>gutenberg</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>austen-persuasion.txt</t>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">When any two young people
-take it into their heads to marry, they are pretty sure by perseverance
-to carry their point, be they ever so poor, or ever so imprudent,
-or ever so little likely to be necessary to each other's ultimate comfort.
-</t>
+          <t>They had just reached the head of the stairs when it seemed, as far as the thickness of the walls would allow them to judge, that a carriage was driving up to the door, and the next moment confirmed the idea by the loud noise of the house-bell.</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>NLTK Gutenberg</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Northanger Abbey.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Leaning back in one corner of the carriage, in a violent burst of tears, she was conveyed some miles beyond the walls of the abbey before she raised her head; and the highest point of ground within the park was almost closed from her view before she was capable of turning her eyes towards it.</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>NLTK Gutenberg</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Northanger Abbey.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>The hope of meeting again in the course of a few years could only put into Catherineâs head what might happen within that time to make a meeting dreadful to her.</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>NLTK Gutenberg</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Northanger Abbey.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Your head runs too much upon Bath; but there is a time for everythingâa time for balls and plays, and a time for work.</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>NLTK Gutenberg</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Northanger Abbey.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>You have had a long run of amusement, and now you must try to be useful.â  Catherine took up her work directly, saying, in a dejected voice, that âher head did not run upon Bathâmuch.â  âThen you are fretting about General Tilney, and that is very simple of you; for ten to one whether you ever see him again.</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>NLTK Gutenberg</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Northanger Abbey.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>CHAPTER 31   Mr. and Mrs. Morlandâs surprise on being applied to by Mr. Tilney for their consent to his marrying their daughter was, for a few minutes, considerable, it having never entered their heads to suspect an attachment on either side; but as nothing, after all, could be more natural than Catherineâs being beloved, they soon learnt to consider it with only the happy agitation of gratified pride, and, as far as they alone were concerned, had not a single objection to start.</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
           <t>heads</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>head</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>head</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>body part</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>english</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>gutenberg</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>austen-persuasion.txt</t>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>body part</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>english</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>NLTK Gutenberg</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Northanger Abbey.txt</t>
         </is>
       </c>
     </row>

</xml_diff>